<commit_message>
Atualiza dados automáticos do Tracker
</commit_message>
<xml_diff>
--- a/dados_tracker/tracker_dados.xlsx
+++ b/dados_tracker/tracker_dados.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Mapas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Agentes'!$A$1:$A$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Agentes'!$A$1:$U$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mapas'!$A$1:$Q$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,17 +429,1440 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n"/>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Funcao</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Time Played</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Win %</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>K/D</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ADR</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ACS</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>DDΔ</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>HS%</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>KAST</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Kills</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Deaths</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Assists</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Attack W/L</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Attack Win %</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Attack K/D</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Defense W/L</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Defense Win %</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Defense K/D</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Clove</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>33 hrs</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>63</v>
+      </c>
+      <c r="F2" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="H2" t="n">
+        <v>153.5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>231</v>
+      </c>
+      <c r="J2" t="n">
+        <v>-12</v>
+      </c>
+      <c r="K2" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="L2" t="n">
+        <v>73.7</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1053</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1185</v>
+      </c>
+      <c r="O2" t="n">
+        <v>475</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>324 - 324</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>50</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>328 - 352</t>
+        </is>
+      </c>
+      <c r="T2" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Jett</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Duelist</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>15 hrs</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>28</v>
+      </c>
+      <c r="F3" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="H3" t="n">
+        <v>146.9</v>
+      </c>
+      <c r="I3" t="n">
+        <v>218.9</v>
+      </c>
+      <c r="J3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="L3" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="M3" t="n">
+        <v>464</v>
+      </c>
+      <c r="N3" t="n">
+        <v>494</v>
+      </c>
+      <c r="O3" t="n">
+        <v>103</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>134 - 176</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>168 - 139</t>
+        </is>
+      </c>
+      <c r="T3" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="U3" t="n">
+        <v>1.14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Sova</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Initiator</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>8.6 hrs</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>16</v>
+      </c>
+      <c r="F4" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="H4" t="n">
+        <v>136.7</v>
+      </c>
+      <c r="I4" t="n">
+        <v>195.1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>-4</v>
+      </c>
+      <c r="K4" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="L4" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="M4" t="n">
+        <v>224</v>
+      </c>
+      <c r="N4" t="n">
+        <v>255</v>
+      </c>
+      <c r="O4" t="n">
+        <v>110</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>75 - 103</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>94 - 72</t>
+        </is>
+      </c>
+      <c r="T4" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Chamber</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>7.3 hrs</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>14</v>
+      </c>
+      <c r="F5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="H5" t="n">
+        <v>123.6</v>
+      </c>
+      <c r="I5" t="n">
+        <v>185.3</v>
+      </c>
+      <c r="J5" t="n">
+        <v>-18</v>
+      </c>
+      <c r="K5" t="n">
+        <v>30</v>
+      </c>
+      <c r="L5" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="M5" t="n">
+        <v>192</v>
+      </c>
+      <c r="N5" t="n">
+        <v>230</v>
+      </c>
+      <c r="O5" t="n">
+        <v>37</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>66 - 87</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>76 - 64</t>
+        </is>
+      </c>
+      <c r="T5" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Duelist</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>3.3 hrs</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="H6" t="n">
+        <v>122.7</v>
+      </c>
+      <c r="I6" t="n">
+        <v>174.8</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-52</v>
+      </c>
+      <c r="K6" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="M6" t="n">
+        <v>82</v>
+      </c>
+      <c r="N6" t="n">
+        <v>115</v>
+      </c>
+      <c r="O6" t="n">
+        <v>32</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>32 - 46</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>41</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>32 - 30</t>
+        </is>
+      </c>
+      <c r="T6" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Neon</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Duelist</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>3.3 hrs</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" t="n">
+        <v>50</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>140.1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>220.1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-3</v>
+      </c>
+      <c r="K7" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="L7" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="M7" t="n">
+        <v>100</v>
+      </c>
+      <c r="N7" t="n">
+        <v>100</v>
+      </c>
+      <c r="O7" t="n">
+        <v>23</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>41 - 28</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="R7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>27 - 36</t>
+        </is>
+      </c>
+      <c r="T7" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="U7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Reyna</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Duelist</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>3.3 hrs</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F8" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="H8" t="n">
+        <v>112.9</v>
+      </c>
+      <c r="I8" t="n">
+        <v>169.2</v>
+      </c>
+      <c r="J8" t="n">
+        <v>-46</v>
+      </c>
+      <c r="K8" t="n">
+        <v>34</v>
+      </c>
+      <c r="L8" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="M8" t="n">
+        <v>75</v>
+      </c>
+      <c r="N8" t="n">
+        <v>121</v>
+      </c>
+      <c r="O8" t="n">
+        <v>24</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>26 - 48</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>22 - 40</t>
+        </is>
+      </c>
+      <c r="T8" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Fade</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Initiator</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2.4 hrs</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H9" t="n">
+        <v>134.5</v>
+      </c>
+      <c r="I9" t="n">
+        <v>193.6</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>+11</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="L9" t="n">
+        <v>77.90000000000001</v>
+      </c>
+      <c r="M9" t="n">
+        <v>62</v>
+      </c>
+      <c r="N9" t="n">
+        <v>65</v>
+      </c>
+      <c r="O9" t="n">
+        <v>29</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>21 - 28</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="R9" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>28 - 18</t>
+        </is>
+      </c>
+      <c r="T9" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Harbor</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1.1 hrs</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>50</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="H10" t="n">
+        <v>114.6</v>
+      </c>
+      <c r="I10" t="n">
+        <v>163.8</v>
+      </c>
+      <c r="J10" t="n">
+        <v>-45</v>
+      </c>
+      <c r="K10" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="L10" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="M10" t="n">
+        <v>26</v>
+      </c>
+      <c r="N10" t="n">
+        <v>36</v>
+      </c>
+      <c r="O10" t="n">
+        <v>23</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>9 - 12</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>12 - 12</t>
+        </is>
+      </c>
+      <c r="T10" t="n">
+        <v>50</v>
+      </c>
+      <c r="U10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cypher</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1.0 hrs</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" t="n">
+        <v>100</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="H11" t="n">
+        <v>133.4</v>
+      </c>
+      <c r="I11" t="n">
+        <v>206.3</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>+8</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="L11" t="n">
+        <v>77.3</v>
+      </c>
+      <c r="M11" t="n">
+        <v>32</v>
+      </c>
+      <c r="N11" t="n">
+        <v>30</v>
+      </c>
+      <c r="O11" t="n">
+        <v>10</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>12 - 8</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>60</v>
+      </c>
+      <c r="R11" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>14 - 10</t>
+        </is>
+      </c>
+      <c r="T11" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="U11" t="n">
+        <v>1.12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Raze</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Duelist</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0.7 hrs</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="n">
+        <v>50</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H12" t="n">
+        <v>167.5</v>
+      </c>
+      <c r="I12" t="n">
+        <v>244.5</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>+13</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="L12" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="M12" t="n">
+        <v>26</v>
+      </c>
+      <c r="N12" t="n">
+        <v>29</v>
+      </c>
+      <c r="O12" t="n">
+        <v>7</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>9 - 11</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>45</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>8 - 5</t>
+        </is>
+      </c>
+      <c r="T12" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="U12" t="n">
+        <v>1.18</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Killjoy</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>0.5 hrs</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>100</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="H13" t="n">
+        <v>200.1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>274.2</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>+79</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="L13" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="M13" t="n">
+        <v>23</v>
+      </c>
+      <c r="N13" t="n">
+        <v>14</v>
+      </c>
+      <c r="O13" t="n">
+        <v>2</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>6 - 5</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>7 - 5</t>
+        </is>
+      </c>
+      <c r="T13" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="U13" t="n">
+        <v>2.67</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Omen</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>0.4 hrs</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>100</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="H14" t="n">
+        <v>221.3</v>
+      </c>
+      <c r="I14" t="n">
+        <v>312.4</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>+68</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="L14" t="n">
+        <v>70</v>
+      </c>
+      <c r="M14" t="n">
+        <v>21</v>
+      </c>
+      <c r="N14" t="n">
+        <v>16</v>
+      </c>
+      <c r="O14" t="n">
+        <v>7</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>7 - 1</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="R14" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>6 - 6</t>
+        </is>
+      </c>
+      <c r="T14" t="n">
+        <v>50</v>
+      </c>
+      <c r="U14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Waylay</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Duelist</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0.4 hrs</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="H15" t="n">
+        <v>106.1</v>
+      </c>
+      <c r="I15" t="n">
+        <v>159.3</v>
+      </c>
+      <c r="J15" t="n">
+        <v>-47</v>
+      </c>
+      <c r="K15" t="n">
+        <v>48</v>
+      </c>
+      <c r="L15" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="M15" t="n">
+        <v>10</v>
+      </c>
+      <c r="N15" t="n">
+        <v>16</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>0 - 6</t>
+        </is>
+      </c>
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>5 - 7</t>
+        </is>
+      </c>
+      <c r="T15" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sage</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0.3 hrs</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>100</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="H16" t="n">
+        <v>197.6</v>
+      </c>
+      <c r="I16" t="n">
+        <v>286.3</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>+88</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="L16" t="n">
+        <v>93.8</v>
+      </c>
+      <c r="M16" t="n">
+        <v>18</v>
+      </c>
+      <c r="N16" t="n">
+        <v>7</v>
+      </c>
+      <c r="O16" t="n">
+        <v>7</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>9 - 3</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>75</v>
+      </c>
+      <c r="R16" t="n">
+        <v>2</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>4 - 0</t>
+        </is>
+      </c>
+      <c r="T16" t="n">
+        <v>100</v>
+      </c>
+      <c r="U16" t="n">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A1"/>
+  <autoFilter ref="A1:U16"/>
+  <conditionalFormatting sqref="F2:F16">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G16">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H16">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I16">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:J16">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K2:K16">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L16">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q2:Q16">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R2:R16">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T2:T16">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U2:U16">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>